<commit_message>
docs(bd): actualizar diccionario de datos con columnas de notificaciones
Registra los campos de control de eventos, carga de envío, referencias, identificador del proveedor y control de reintentos de la tabla notificacion.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Modelo de Datos/diccionario de datos SIGET.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Modelo de Datos/diccionario de datos SIGET.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario de datos SIGET" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diccionario de datos SIGET'!$A$1:$J$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diccionario de datos SIGET'!$A$1:$J$211</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J204"/>
+  <dimension ref="A1:J211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -9487,8 +9487,198 @@
         </is>
       </c>
     </row>
+    <row r="205" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A205" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B205" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C205" s="2" t="str">
+        <v>14</v>
+      </c>
+      <c r="D205" s="2" t="str">
+        <v>clave_evento</v>
+      </c>
+      <c r="E205" s="2" t="str">
+        <v>character varying(255)</v>
+      </c>
+      <c r="F205" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="G205" s="2" t="str">
+        <v>UNIQUE</v>
+      </c>
+      <c r="H205" s="2"/>
+      <c r="I205" s="2"/>
+      <c r="J205" s="2" t="str">
+        <v>Identificador único del evento de negocio para evitar avisos duplicados. El índice uq_notificacion_clave_evento permite varios valores NULL.</v>
+      </c>
+    </row>
+    <row r="206" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A206" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B206" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C206" s="2" t="str">
+        <v>15</v>
+      </c>
+      <c r="D206" s="2" t="str">
+        <v>datos_envio</v>
+      </c>
+      <c r="E206" s="2" t="str">
+        <v>jsonb</v>
+      </c>
+      <c r="F206" s="2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="G206" s="2"/>
+      <c r="H206" s="2"/>
+      <c r="I206" s="2" t="str">
+        <v>'{}'::jsonb</v>
+      </c>
+      <c r="J206" s="2" t="str">
+        <v>Contenido del correo fijado al registrar el aviso. Los reintentos conservan el remitente, destinatarios, asunto y cuerpo originales.</v>
+      </c>
+    </row>
+    <row r="207" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A207" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B207" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C207" s="2" t="str">
+        <v>16</v>
+      </c>
+      <c r="D207" s="2" t="str">
+        <v>referencia</v>
+      </c>
+      <c r="E207" s="2" t="str">
+        <v>jsonb</v>
+      </c>
+      <c r="F207" s="2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="G207" s="2"/>
+      <c r="H207" s="2"/>
+      <c r="I207" s="2" t="str">
+        <v>'{}'::jsonb</v>
+      </c>
+      <c r="J207" s="2" t="str">
+        <v>Datos del registro de negocio asociado al aviso, utilizados para comprobar su vigencia antes del envío.</v>
+      </c>
+    </row>
+    <row r="208" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A208" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B208" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C208" s="2" t="str">
+        <v>17</v>
+      </c>
+      <c r="D208" s="2" t="str">
+        <v>id_proveedor</v>
+      </c>
+      <c r="E208" s="2" t="str">
+        <v>character varying(100)</v>
+      </c>
+      <c r="F208" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="G208" s="2"/>
+      <c r="H208" s="2"/>
+      <c r="I208" s="2"/>
+      <c r="J208" s="2" t="str">
+        <v>Identificador del mensaje aceptado por el proveedor externo, utilizado para consultar su entrega.</v>
+      </c>
+    </row>
+    <row r="209" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A209" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B209" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C209" s="2" t="str">
+        <v>18</v>
+      </c>
+      <c r="D209" s="2" t="str">
+        <v>reintento_permitido</v>
+      </c>
+      <c r="E209" s="2" t="str">
+        <v>boolean</v>
+      </c>
+      <c r="F209" s="2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="G209" s="2"/>
+      <c r="H209" s="2"/>
+      <c r="I209" s="2" t="str">
+        <v>true</v>
+      </c>
+      <c r="J209" s="2" t="str">
+        <v>Indica si el aviso admite otro intento de envío cuando se cumplen los límites y la espera configurados.</v>
+      </c>
+    </row>
+    <row r="210" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A210" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B210" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C210" s="2" t="str">
+        <v>19</v>
+      </c>
+      <c r="D210" s="2" t="str">
+        <v>proximo_intento</v>
+      </c>
+      <c r="E210" s="2" t="str">
+        <v>timestamp with time zone</v>
+      </c>
+      <c r="F210" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="G210" s="2"/>
+      <c r="H210" s="2"/>
+      <c r="I210" s="2"/>
+      <c r="J210" s="2" t="str">
+        <v>Fecha y hora a partir de las cuales puede realizarse el siguiente intento de envío.</v>
+      </c>
+    </row>
+    <row r="211" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A211" s="2" t="str">
+        <v>07 - QR, notificaciones y auditoría</v>
+      </c>
+      <c r="B211" s="2" t="str">
+        <v>notificacion</v>
+      </c>
+      <c r="C211" s="2" t="str">
+        <v>20</v>
+      </c>
+      <c r="D211" s="2" t="str">
+        <v>fecha_primer_intento</v>
+      </c>
+      <c r="E211" s="2" t="str">
+        <v>timestamp with time zone</v>
+      </c>
+      <c r="F211" s="2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="G211" s="2"/>
+      <c r="H211" s="2"/>
+      <c r="I211" s="2"/>
+      <c r="J211" s="2" t="str">
+        <v>Fecha y hora del primer intento de envío, utilizada para controlar la ventana de idempotencia.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J204"/>
+  <autoFilter ref="A1:J211"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>